<commit_message>
Add new gaming projects 9-16 from spreadsheet and fix folder names
</commit_message>
<xml_diff>
--- a/img/game links.xlsx
+++ b/img/game links.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/muneebiftikhar/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/DataDrive/Websites/portfolio/img/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{42C01719-3220-0A43-9374-252F47F4FE03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0E4F46E-68A8-4F4F-B2CD-354DA9A77678}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2380" yWindow="1880" windowWidth="28040" windowHeight="17440" xr2:uid="{EE73593E-7F94-C84D-87C4-ACA4BDA8DEE0}"/>
+    <workbookView xWindow="80" yWindow="500" windowWidth="33600" windowHeight="19400" xr2:uid="{EE73593E-7F94-C84D-87C4-ACA4BDA8DEE0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
   <si>
     <t xml:space="preserve">Game Link </t>
   </si>
@@ -89,6 +89,54 @@
   </si>
   <si>
     <t>/Volumes/DataDrive/Websites/portfolio/img/BSWRM_Sim</t>
+  </si>
+  <si>
+    <t>https://play.google.com/store/apps/details?id=com.ozipub.crazy.doctor&amp;pcampaignid=web_share</t>
+  </si>
+  <si>
+    <t>/Volumes/DataDrive/Websites/portfolio/img/crzyDoctor</t>
+  </si>
+  <si>
+    <t>https://play.google.com/store/apps/details?id=com.merge.battle.fight.heroes.games&amp;pcampaignid=web_share</t>
+  </si>
+  <si>
+    <t>/Volumes/DataDrive/Websites/portfolio/img/spinBattle</t>
+  </si>
+  <si>
+    <t>https://play.google.com/store/apps/details?id=com.bonebreaker.ragdoll.race.game.simulator&amp;pcampaignid=web_share</t>
+  </si>
+  <si>
+    <t>/Volumes/DataDrive/Websites/portfolio/img/radDoll</t>
+  </si>
+  <si>
+    <t>https://play.google.com/store/apps/details?id=com.yhi.punch.smash.boxing.arms&amp;pcampaignid=web_share</t>
+  </si>
+  <si>
+    <t>Volumes/DataDrive/Websites/portfolio/img/punchitt </t>
+  </si>
+  <si>
+    <t>https://play.google.com/store/apps/details?id=com.sling.strike.action.whackgame.simulator&amp;pcampaignid=web_share</t>
+  </si>
+  <si>
+    <t>/Volumes/DataDrive/Websites/portfolio/img/slingShott</t>
+  </si>
+  <si>
+    <t>https://play.google.com/store/apps/details?id=com.scary.mom.bad.cat.pet.simulator.games&amp;pcampaignid=web_share</t>
+  </si>
+  <si>
+    <t>/Volumes/DataDrive/Websites/portfolio/img/Bad_Cat</t>
+  </si>
+  <si>
+    <t>https://play.google.com/store/apps/details?id=com.toy.soldiers.fps.war.battle.shooting&amp;pcampaignid=web_share</t>
+  </si>
+  <si>
+    <t>/Volumes/DataDrive/Websites/portfolio/img/plasticArmy</t>
+  </si>
+  <si>
+    <t>https://play.google.com/store/apps/details?id=com.g247.spiral.ramp.car.racing.stunt.game&amp;pcampaignid=web_share</t>
+  </si>
+  <si>
+    <t>/Volumes/DataDrive/Websites/portfolio/img/idlecar</t>
   </si>
 </sst>
 </file>
@@ -465,7 +513,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E6181C9-79F7-A94E-A731-AB2BDB155119}">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="103.33203125" customWidth="1"/>
@@ -542,6 +590,70 @@
       </c>
       <c r="B9" s="3" t="s">
         <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="43" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A13" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A16" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A17" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -554,6 +666,14 @@
     <hyperlink ref="A7" r:id="rId6" xr:uid="{B73176F9-DE55-2D42-A846-05768F7FEE66}"/>
     <hyperlink ref="A8" r:id="rId7" xr:uid="{6BAABCA3-07B8-714C-B366-ED1684A0890E}"/>
     <hyperlink ref="A9" r:id="rId8" xr:uid="{22D18D63-1C0D-BA44-87DE-F21F14441E47}"/>
+    <hyperlink ref="A10" r:id="rId9" xr:uid="{CEDB75FC-7BA9-E043-8C1A-25835F4EE6A9}"/>
+    <hyperlink ref="A15" r:id="rId10" xr:uid="{6B8022F9-86E8-8142-A41E-28EA32FB45D5}"/>
+    <hyperlink ref="A12" r:id="rId11" xr:uid="{0478E5EE-932B-8C46-A81F-17D6595361C5}"/>
+    <hyperlink ref="A13" r:id="rId12" xr:uid="{A2AEEBA2-A1EA-3742-BC6A-0B05448A9E9A}"/>
+    <hyperlink ref="A14" r:id="rId13" xr:uid="{C272B26B-715A-FB43-8D1E-4F858DBEA6FF}"/>
+    <hyperlink ref="A11" r:id="rId14" xr:uid="{12ADF184-65A8-EB45-B263-F67AB4880475}"/>
+    <hyperlink ref="A16" r:id="rId15" xr:uid="{0E029976-0B26-9040-A858-F21F3DC5E25A}"/>
+    <hyperlink ref="A17" r:id="rId16" xr:uid="{29E7A83D-0342-0B4C-BEA0-1E5EC87C9944}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>